<commit_message>
create table usertoken + add refeshtoken feature
</commit_message>
<xml_diff>
--- a/Movie24hDB.xlsx
+++ b/Movie24hDB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1.ProgrammingLanguage\ASP.NET Core\Movie24h\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D908EC-B87E-4299-B19D-E7CFDF03ACED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D55C45F-5C87-4D21-8507-DAAA0FCD3E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="65">
   <si>
     <t>MemberId</t>
   </si>
@@ -78,21 +78,12 @@
     <t>PRI</t>
   </si>
   <si>
-    <t>VARCHAR(100)</t>
-  </si>
-  <si>
     <t>FullName</t>
   </si>
   <si>
-    <t>CHAR(100)</t>
-  </si>
-  <si>
     <t>Address</t>
   </si>
   <si>
-    <t>VARCHAR(200)</t>
-  </si>
-  <si>
     <t>FOR</t>
   </si>
   <si>
@@ -114,9 +105,6 @@
     <t>PhoneNumber</t>
   </si>
   <si>
-    <t>CHAR(10)</t>
-  </si>
-  <si>
     <t>Email</t>
   </si>
   <si>
@@ -126,9 +114,6 @@
     <t>Fax</t>
   </si>
   <si>
-    <t>CHAR(20)</t>
-  </si>
-  <si>
     <t>CreateDate</t>
   </si>
   <si>
@@ -138,9 +123,6 @@
     <t>CCCD</t>
   </si>
   <si>
-    <t>CHAR(12)</t>
-  </si>
-  <si>
     <t>CreateById</t>
   </si>
   <si>
@@ -180,9 +162,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>VARCHAR(500)</t>
-  </si>
-  <si>
     <t>Gender</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -215,7 +194,67 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>CHAR(36)</t>
+    <t>USERTOKEN</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>FOR</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>RefreshToken</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(500)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(100)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(200)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(10)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(20)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(12)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(36)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NVARCHAR(MAX)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Expiration</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>DeviceInfo</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>IP</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>RevokedDate</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>CreateDate</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -223,7 +262,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,6 +280,15 @@
     </font>
     <font>
       <sz val="6"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="游ゴシック"/>
       <family val="3"/>
       <charset val="128"/>
@@ -267,7 +315,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -290,11 +338,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -325,6 +388,22 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,30 +781,38 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FD7B499-A7AD-4799-BD2A-56723A349D3F}">
-  <dimension ref="B2:N29"/>
+  <dimension ref="B2:U29"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="4.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.125" customWidth="1"/>
+    <col min="17" max="17" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P2" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
@@ -762,8 +849,26 @@
       <c r="N3" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B4" s="2">
         <v>1</v>
       </c>
@@ -771,7 +876,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>12</v>
@@ -784,10 +889,10 @@
         <v>1</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>12</v>
@@ -796,16 +901,32 @@
         <v>1</v>
       </c>
       <c r="N4" s="3"/>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P4" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="U4" s="3"/>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B5" s="2">
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="4" t="b">
@@ -816,26 +937,42 @@
         <v>2</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P5" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="T5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" s="3"/>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B6" s="2">
         <v>3</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="4" t="b">
@@ -846,28 +983,42 @@
         <v>3</v>
       </c>
       <c r="J6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" s="3"/>
+      <c r="P6" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="M6" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="R6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="S6" s="2"/>
+      <c r="T6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" s="3"/>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B7" s="2">
         <v>4</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="4" t="b">
@@ -878,28 +1029,42 @@
         <v>4</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M7" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N7" s="3"/>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P7" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="2"/>
+      <c r="T7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" s="3"/>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B8" s="2">
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="4" t="b">
@@ -910,28 +1075,42 @@
         <v>5</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M8" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N8" s="3"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P8" s="2">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="S8" s="2"/>
+      <c r="T8" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U8" s="3"/>
+    </row>
+    <row r="9" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B9" s="2">
         <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="4" t="b">
@@ -942,28 +1121,42 @@
         <v>6</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M9" s="9" t="b">
         <v>0</v>
       </c>
       <c r="N9" s="8"/>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P9" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="R9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="S9" s="2"/>
+      <c r="T9" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U9" s="3"/>
+    </row>
+    <row r="10" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B10" s="2">
         <v>7</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="4" t="b">
@@ -974,26 +1167,40 @@
         <v>7</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P10" s="2">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="S10" s="2"/>
+      <c r="T10" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U10" s="3"/>
+    </row>
+    <row r="11" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B11" s="2">
         <v>8</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="4" t="b">
@@ -1004,26 +1211,40 @@
         <v>8</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P11" s="11">
+        <v>8</v>
+      </c>
+      <c r="Q11" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="R11" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="S11" s="11"/>
+      <c r="T11" s="13" t="b">
+        <v>0</v>
+      </c>
+      <c r="U11" s="12"/>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B12" s="2">
         <v>9</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="4" t="b">
@@ -1034,26 +1255,32 @@
         <v>9</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P12" s="14"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="14"/>
+      <c r="T12" s="15"/>
+      <c r="U12" s="15"/>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B13" s="2">
         <v>10</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="4" t="b">
@@ -1064,165 +1291,213 @@
         <v>10</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P13" s="14"/>
+      <c r="Q13" s="15"/>
+      <c r="R13" s="15"/>
+      <c r="S13" s="14"/>
+      <c r="T13" s="15"/>
+      <c r="U13" s="15"/>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B14" s="2">
         <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F14" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I14" s="2">
         <v>11</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N14" s="3"/>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P14" s="14"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="14"/>
+      <c r="T14" s="15"/>
+      <c r="U14" s="15"/>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B15" s="2">
         <v>12</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F15" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="15"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="15"/>
+      <c r="U15" s="15"/>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B16" s="2">
         <v>13</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F16" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I16" s="6"/>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P16" s="14"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="14"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+    </row>
+    <row r="17" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B17" s="2">
         <v>14</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G17" s="3"/>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P17" s="14"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="14"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+    </row>
+    <row r="18" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B18" s="2">
         <v>15</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G18" s="3"/>
-    </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P18" s="14"/>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="15"/>
+      <c r="U18" s="15"/>
+    </row>
+    <row r="19" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B19" s="2">
         <v>16</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G19" s="3"/>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P19" s="14"/>
+      <c r="Q19" s="15"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="14"/>
+      <c r="T19" s="15"/>
+      <c r="U19" s="15"/>
+    </row>
+    <row r="20" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B20" s="2">
         <v>17</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="4" t="b">
         <v>0</v>
       </c>
       <c r="G20" s="3"/>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.4">
+      <c r="P20" s="14"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="14"/>
+      <c r="T20" s="15"/>
+      <c r="U20" s="15"/>
+    </row>
+    <row r="24" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B24" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B25" s="5" t="s">
         <v>5</v>
       </c>
@@ -1260,7 +1535,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B26" s="2">
         <v>1</v>
       </c>
@@ -1268,7 +1543,7 @@
         <v>11</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>12</v>
@@ -1282,7 +1557,7 @@
         <v>11</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>12</v>
@@ -1292,15 +1567,15 @@
       </c>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B27" s="2">
         <v>2</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="4" t="b">
@@ -1309,10 +1584,10 @@
       <c r="G27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="4" t="b">
@@ -1320,15 +1595,15 @@
       </c>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:21" x14ac:dyDescent="0.4">
       <c r="B28" s="2">
         <v>3</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="4" t="b">
@@ -1337,26 +1612,26 @@
       <c r="G28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M28" s="4" t="b">
         <v>0</v>
       </c>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:21" x14ac:dyDescent="0.4">
       <c r="I29" s="3"/>
       <c r="J29" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="L29" s="3"/>
       <c r="M29" s="4" t="b">

</xml_diff>